<commit_message>
XLSX: outstanding students destinations + pubs
</commit_message>
<xml_diff>
--- a/xlsx/site.xlsx
+++ b/xlsx/site.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'people'!$A$1:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'people'!$A$1:$O$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'publications'!$A$1:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'projects'!$A$1:$K$10</definedName>
   </definedNames>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,10 +475,25 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>destination_en</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>destination_zh</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>pub_ids</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>is_outstanding</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>outstanding_order</t>
         </is>
@@ -505,6 +520,21 @@
           <t>区宝文</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>iccad-2025-astra</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -527,6 +557,21 @@
           <t>刘博豪</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>dac-2026-openacmv2</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -549,12 +594,33 @@
           <t>戴国浩</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
+          <t>HKUST(GZ)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>港科广</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>aspdac-2023-entropy-reduction;dac-2023-yield-barrier;iccad-2023-opt;ijhe-2023-sofc</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -579,11 +645,25 @@
           <t>刘佳展</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>/people/jiazhan_liu.png</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>dac-2026-breaking-tuning-barrier</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -606,6 +686,17 @@
           <t>商靖海</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -628,11 +719,21 @@
           <t>王继熠</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>/people/jiyi_wang.png</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -655,6 +756,21 @@
           <t>黄凯期</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>dac-2025-exploiting;dac-2026-breaking-tuning-barrier;iseda-2026-portable</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -677,11 +793,21 @@
           <t>廖宏商</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>/people/hongshang_liao.png</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -704,6 +830,17 @@
           <t>林伟斌</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -726,6 +863,17 @@
           <t>麦梓睿</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -748,6 +896,21 @@
           <t>梅沁心</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>dac-2025-exploiting;dac-2026-openacmv2;iseda-2026-portable</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -770,6 +933,17 @@
           <t>唐浩浩</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -802,6 +976,7 @@
           <t>导师</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>/people/wei.png</t>
@@ -817,6 +992,15 @@
           <t>英国谢菲尔德大学数学与统计学院讲师，华威大学博士，前北京航空航天大学助理教授。研究成果发表于 Nature 子刊、NeurIPS、DAC、ICCAD、AAAI、TODAES 等顶级会议与期刊，2025 年入选英国 Manchester Prize 十强。已指导多名深大本科生直博北京大学、北京航空航天大学、香港科技大学等高校。</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>dac-2026-openacmv2;dac-2024-every-failure;iccad-2024-aro</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -839,12 +1023,33 @@
           <t>范炜建</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
+          <t>PhD at Peking University</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>北京大学直博</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>dac-2024-every-failure;dac-2024-kato</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="O15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -869,6 +1074,21 @@
           <t>谢炜伦</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>iccad-2025-dive;iseda-2025-design-space-folding</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -891,6 +1111,17 @@
           <t>周熙曦</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -913,6 +1144,17 @@
           <t>徐一鹏</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -935,6 +1177,17 @@
           <t>苑艺钟</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -957,11 +1210,21 @@
           <t>朱则熹</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>/people/zexi_zhu.png</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -984,6 +1247,17 @@
           <t>招俊安</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1006,12 +1280,33 @@
           <t>卢振杰</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
+          <t>Southern University of Science and Technology</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>南方科技大学</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>iccad-2024-aro</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1036,17 +1331,38 @@
           <t>刘卓铧</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
+          <t>PhD at Beihang University</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>北京航空航天大学直博</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>dac-2025-exploiting;dac-2026-openacmv2;iseda-2026-portable;iccad-2025-astra;iccad-2025-dive;iccd-2025-openyield;iseda-2025-design-space-folding;dac-2024-kato</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="L23" t="n">
+      <c r="O23" t="n">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
+  <autoFilter ref="A1:O23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1141,6 +1457,8 @@
           <t>https://arxiv.org/abs/2512.00712</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1176,6 +1494,8 @@
           <t>#</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1211,6 +1531,8 @@
           <t>#</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1238,7 +1560,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Zhuohua Liu鈥?;Kaiqi Huang鈥?;qinxin-mei;Yuanqi Hu;Wei W. Xing</t>
+          <t>zhuohua-liu;kaiqi-huang;qinxin-mei;Yuanqi Hu;Wei W. Xing</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1246,6 +1568,8 @@
           <t>#</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1281,6 +1605,8 @@
           <t>https://doi.org/10.1021/acs.est.5c07557</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1316,6 +1642,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/11240675/</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1351,6 +1679,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/11240976/</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1386,6 +1716,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/11310974/</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1421,6 +1753,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/11100880/</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1456,6 +1790,8 @@
           <t>https://doi.org/10.1016/j.procir.2025.01.046</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1491,6 +1827,8 @@
           <t>https://dl.acm.org/doi/abs/10.1145/3649329.3657381</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1526,6 +1864,8 @@
           <t>https://dl.acm.org/doi/abs/10.1145/3649329.3657380</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1561,6 +1901,8 @@
           <t>https://dl.acm.org/doi/abs/10.1145/3676536.3676713</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1596,6 +1938,8 @@
           <t>https://dl.acm.org/doi/abs/10.1145/3566097.3567907</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1631,6 +1975,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/10247952/</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1666,6 +2012,8 @@
           <t>https://ieeexplore.ieee.org/abstract/document/10323689/</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1701,6 +2049,8 @@
           <t>https://www.sciencedirect.com/science/article/pii/S0360319923017007</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I18"/>
@@ -1825,6 +2175,7 @@
           <t>利用神经算子学习偏微分方程的映射。</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1877,6 +2228,7 @@
           <t>整理并开源 EDA 良率算法，后续加入良率算法开发。</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1929,6 +2281,7 @@
           <t>整理并开源 EDA 优化算法，后续加入优化算法开发。</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1981,6 +2334,7 @@
           <t>基于 LLM 从非结构化 EPD 中抽取关键环境指标（如 GWP），构建结构化知识库。</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2033,6 +2387,7 @@
           <t>结合大模型与微调小模型预测 ecoinvent 表格数值，并扩展到更多未知数据集。</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2085,6 +2440,7 @@
           <t>基于 LLM Agent 的端到端自动化流程：BOM 解析、数据库检索匹配（如 Ecoinvent）、碳排计算与 LCA 报告生成，减少人工干预。</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2137,6 +2493,7 @@
           <t>结合大模型智能体与运筹优化，将 LCA 从物料清单分析扩展到绿色材料替代的端到端自动化决策。</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2189,6 +2546,7 @@
           <t>使用 AI 辅助 LCI 清单的组件与环境数据库（如 Ecoinvent）中的名称与活动进行匹配。</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2241,6 +2599,7 @@
           <t>面向良率的 sizing 优化。</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K10"/>

</xml_diff>